<commit_message>
Updated annotations and added mcp based taxonomy analysis
</commit_message>
<xml_diff>
--- a/annotations/llm-scheduler-single-trajectory.xlsx
+++ b/annotations/llm-scheduler-single-trajectory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Studies\UZH-M.Sc\THESIS\demo_v1\outputs\2026-08-25_claude_fable_single_trajectory\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Studies\UZH-M.Sc\THESIS\design-decisions-by-LLMs\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6602A6-3982-4CA0-B6D5-D1B9EB18A67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB376430-B53E-46D5-B57D-7B235307A8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trajectory Steps" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="162">
   <si>
     <t>Single Trajectory Annotation — Claude Fable 5 + Claude Code</t>
   </si>
@@ -1871,6 +1871,28 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1922,33 +1944,11 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="26">
     <dxf>
       <font>
         <b/>
@@ -2285,19 +2285,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="20"/>
-        <color rgb="FF1F2937"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2312,16 +2299,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrajectoryStepsTable" displayName="TrajectoryStepsTable" ref="A13:I26" totalsRowShown="0" dataDxfId="26">
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Step" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Thought" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Action" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Observation" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Decision?" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Event ID" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Primary category" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Primary reason" dataDxfId="18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TrajectoryStepsTable" displayName="TrajectoryStepsTable" ref="A13:H26" totalsRowShown="0" dataDxfId="25">
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Step" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Thought" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Action" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Observation" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Decision?" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Event ID" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Primary category" dataDxfId="18"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Decision summary" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2546,7 +2532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="39.59765625" customWidth="1"/>
@@ -2555,102 +2541,97 @@
     <col min="4" max="4" width="58" customWidth="1"/>
     <col min="5" max="5" width="39.3984375" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="34.59765625" customWidth="1"/>
-    <col min="10" max="10" width="38" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="34.59765625" customWidth="1"/>
+    <col min="9" max="9" width="38" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28.05" customHeight="1">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:11" ht="28.05" customHeight="1">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-    </row>
-    <row r="3" spans="1:12" ht="22.8">
-      <c r="A3" s="59" t="s">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+    </row>
+    <row r="3" spans="1:11" ht="22.8">
+      <c r="A3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="43"/>
-    </row>
-    <row r="4" spans="1:12" ht="22.8">
-      <c r="A4" s="61" t="s">
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="51"/>
+    </row>
+    <row r="4" spans="1:11" ht="22.8">
+      <c r="A4" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="46"/>
-    </row>
-    <row r="5" spans="1:12" ht="22.8">
-      <c r="A5" s="61" t="s">
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="54"/>
+    </row>
+    <row r="5" spans="1:11" ht="22.8">
+      <c r="A5" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="47"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="49"/>
-    </row>
-    <row r="6" spans="1:12" ht="22.8">
-      <c r="A6" s="61" t="s">
+      <c r="D5" s="55"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="57"/>
+    </row>
+    <row r="6" spans="1:11" ht="22.8">
+      <c r="A6" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="52"/>
-    </row>
-    <row r="7" spans="1:12" ht="22.8">
-      <c r="A7" s="61" t="s">
+      <c r="D6" s="58"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="60"/>
+    </row>
+    <row r="7" spans="1:11" ht="22.8">
+      <c r="A7" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="43" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="39"/>
@@ -2661,13 +2642,12 @@
       <c r="I7" s="39"/>
       <c r="J7" s="39"/>
       <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-    </row>
-    <row r="8" spans="1:12" ht="22.8">
-      <c r="A8" s="61" t="s">
+    </row>
+    <row r="8" spans="1:11" ht="22.8">
+      <c r="A8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="66">
+      <c r="B8" s="47">
         <v>13</v>
       </c>
       <c r="D8" s="39"/>
@@ -2678,47 +2658,45 @@
       <c r="I8" s="39"/>
       <c r="J8" s="39"/>
       <c r="K8" s="39"/>
-      <c r="L8" s="39"/>
-    </row>
-    <row r="9" spans="1:12" ht="22.8">
-      <c r="A9" s="61" t="s">
+    </row>
+    <row r="9" spans="1:11" ht="22.8">
+      <c r="A9" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="66">
+      <c r="B9" s="47">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="22.8">
-      <c r="A10" s="63" t="s">
+    <row r="10" spans="1:11" ht="22.8">
+      <c r="A10" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="64" t="s">
+      <c r="B10" s="45" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="22.8">
-      <c r="A11" s="65"/>
-      <c r="B11" s="65"/>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="53" t="s">
+    <row r="11" spans="1:11" ht="22.8">
+      <c r="A11" s="46"/>
+      <c r="B11" s="46"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="56" t="s">
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="57"/>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
-      <c r="I12" s="57"/>
-      <c r="J12" s="57"/>
-      <c r="K12" s="57"/>
-      <c r="L12" s="58"/>
-    </row>
-    <row r="13" spans="1:12" ht="27.6">
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="65"/>
+      <c r="K12" s="66"/>
+    </row>
+    <row r="13" spans="1:11" ht="27.6">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
@@ -2741,13 +2719,10 @@
         <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I13" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="88.05" customHeight="1">
+    <row r="14" spans="1:11" ht="88.05" customHeight="1">
       <c r="A14" s="24">
         <v>0</v>
       </c>
@@ -2764,9 +2739,8 @@
       <c r="F14" s="28"/>
       <c r="G14" s="28"/>
       <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="1:12" ht="88.05" customHeight="1">
+    </row>
+    <row r="15" spans="1:11" ht="88.05" customHeight="1">
       <c r="A15" s="29">
         <v>1</v>
       </c>
@@ -2781,9 +2755,8 @@
       <c r="F15" s="33"/>
       <c r="G15" s="33"/>
       <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
-    </row>
-    <row r="16" spans="1:12" ht="88.05" customHeight="1">
+    </row>
+    <row r="16" spans="1:11" ht="88.05" customHeight="1">
       <c r="A16" s="29">
         <v>2</v>
       </c>
@@ -2800,9 +2773,8 @@
       <c r="F16" s="33"/>
       <c r="G16" s="33"/>
       <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-    </row>
-    <row r="17" spans="1:9" ht="88.05" customHeight="1">
+    </row>
+    <row r="17" spans="1:8" ht="88.05" customHeight="1">
       <c r="A17" s="29">
         <v>3</v>
       </c>
@@ -2819,9 +2791,8 @@
       <c r="F17" s="33"/>
       <c r="G17" s="33"/>
       <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-    </row>
-    <row r="18" spans="1:9" ht="88.05" customHeight="1">
+    </row>
+    <row r="18" spans="1:8" ht="88.05" customHeight="1">
       <c r="A18" s="29">
         <v>4</v>
       </c>
@@ -2844,13 +2815,10 @@
         <v>42</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="I18" s="33" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="88.05" customHeight="1">
+    <row r="19" spans="1:8" ht="88.05" customHeight="1">
       <c r="A19" s="29">
         <v>5</v>
       </c>
@@ -2873,13 +2841,10 @@
         <v>42</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="I19" s="33" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="88.05" customHeight="1">
+    <row r="20" spans="1:8" ht="88.05" customHeight="1">
       <c r="A20" s="29">
         <v>6</v>
       </c>
@@ -2902,13 +2867,10 @@
         <v>42</v>
       </c>
       <c r="H20" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I20" s="33" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="88.05" customHeight="1">
+    <row r="21" spans="1:8" ht="88.05" customHeight="1">
       <c r="A21" s="29">
         <v>7</v>
       </c>
@@ -2931,13 +2893,10 @@
         <v>42</v>
       </c>
       <c r="H21" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I21" s="33" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="88.05" customHeight="1">
+    <row r="22" spans="1:8" ht="88.05" customHeight="1">
       <c r="A22" s="29">
         <v>8</v>
       </c>
@@ -2960,13 +2919,10 @@
         <v>42</v>
       </c>
       <c r="H22" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I22" s="33" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="88.05" customHeight="1">
+    <row r="23" spans="1:8" ht="88.05" customHeight="1">
       <c r="A23" s="29">
         <v>9</v>
       </c>
@@ -2989,13 +2945,10 @@
         <v>65</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="I23" s="33" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="88.05" customHeight="1">
+    <row r="24" spans="1:8" ht="88.05" customHeight="1">
       <c r="A24" s="29">
         <v>10</v>
       </c>
@@ -3018,13 +2971,10 @@
         <v>71</v>
       </c>
       <c r="H24" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="I24" s="33" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="88.05" customHeight="1">
+    <row r="25" spans="1:8" ht="88.05" customHeight="1">
       <c r="A25" s="29">
         <v>11</v>
       </c>
@@ -3047,13 +2997,10 @@
         <v>78</v>
       </c>
       <c r="H25" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="I25" s="33" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="88.05" customHeight="1">
+    <row r="26" spans="1:8" ht="88.05" customHeight="1">
       <c r="A26" s="34">
         <v>12</v>
       </c>
@@ -3072,19 +3019,16 @@
         <v>83</v>
       </c>
       <c r="H26" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="I26" s="38" t="s">
         <v>84</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D3:L3"/>
-    <mergeCell ref="D4:L6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="D4:K6"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E12:L12"/>
+    <mergeCell ref="E12:K12"/>
   </mergeCells>
   <conditionalFormatting sqref="E14:E26">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -3112,23 +3056,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="27.6">
       <c r="A3" s="4" t="s">
@@ -3466,14 +3410,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
@@ -3631,7 +3575,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" ht="27.6">
       <c r="A15" s="9" t="s">
         <v>98</v>
       </c>

</xml_diff>